<commit_message>
feat: implement pediatric baseline calibration, smart alerts, and clinical documentation
</commit_message>
<xml_diff>
--- a/supabase_values.xlsx
+++ b/supabase_values.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\chriz\Desktop\Hikon2.1.1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E042AE27-9B9F-4C4B-AE81-C437C9164BC5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0F0272AD-3C39-4095-B438-55B3BAECEDCE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3312" yWindow="3504" windowWidth="17280" windowHeight="9960" xr2:uid="{F215C3E6-5F85-4129-9234-E5A19808AB2B}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{F215C3E6-5F85-4129-9234-E5A19808AB2B}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="682" uniqueCount="336">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="683" uniqueCount="337">
   <si>
     <t>id</t>
   </si>
@@ -1044,6 +1044,9 @@
   </si>
   <si>
     <t>2026-04-07 20:39:30.976778+00</t>
+  </si>
+  <si>
+    <t>br_rate</t>
   </si>
 </sst>
 </file>
@@ -1422,13 +1425,22 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2E17A204-1E27-4E69-A6EC-D4CAE41E52F3}">
-  <dimension ref="A1:T193"/>
+  <dimension ref="A1:U193"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
+    <col min="1" max="1" width="39.44140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.109375" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="27.77734375" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="10" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.21875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="10" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="14.5546875" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="8.5546875" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="30.21875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="7.5546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1489,18 +1501,21 @@
       <c r="T1" t="s">
         <v>19</v>
       </c>
-    </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.3">
+      <c r="U1" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>27</v>
       </c>
@@ -1547,7 +1562,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>30</v>
       </c>
@@ -1594,7 +1609,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>33</v>
       </c>
@@ -1641,7 +1656,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>36</v>
       </c>
@@ -1688,12 +1703,12 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>39</v>
       </c>
@@ -1740,7 +1755,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:20" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:21" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>42</v>
       </c>
@@ -1787,7 +1802,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>45</v>
       </c>
@@ -1834,12 +1849,12 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
         <v>48</v>
       </c>

</xml_diff>